<commit_message>
Correction du fichier Gantt (valeurs de test retirées)
</commit_message>
<xml_diff>
--- a/01-techniques-de-gestion-de-projets/rendu-de-sousa-nunes-alessandro/projet-2-cahier-charges-gantt/planning-gantt.xlsx
+++ b/01-techniques-de-gestion-de-projets/rendu-de-sousa-nunes-alessandro/projet-2-cahier-charges-gantt/planning-gantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0ee8758c4b754eab/Bureau/E3-Gestion-de-projets-PPE/01-techniques-de-gestion-de-projets/rendu-de-sousa-nunes-alessandro/projet-2-cahier-charges-gantt/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="8_{3A977EDB-7773-4313-8E24-2E865FBDD732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F97A89C-CC36-447C-B27A-EAFF2F9AC0DA}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{3A977EDB-7773-4313-8E24-2E865FBDD732}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB0A6AA2-5C34-4D57-88DE-CE0C2CEB5C77}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{AA88D5F3-5099-4AFB-9E88-DDB1477EE6E8}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
   <si>
     <t>Planning Gantt - Outil de réservation de salles (client : fiduciaire)</t>
   </si>
@@ -193,9 +193,6 @@
   </si>
   <si>
     <t>Légende : rouge = tâche critique (marge 0), bleu = tâche avec marge. Dates, marges et chemin critique sont calculés par formules à partir des durées et des prédécesseurs.</t>
-  </si>
-  <si>
-    <t>TEST 2 : durée de F passée de 7 à 9 jours (fichier non enregistré)</t>
   </si>
 </sst>
 </file>
@@ -250,15 +247,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -268,12 +263,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -320,7 +309,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -349,13 +338,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,6 +379,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1208,7 +1198,7 @@
       <c r="B8" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="14">
         <v>3</v>
       </c>
       <c r="D8" s="10" t="s">
@@ -1232,15 +1222,15 @@
       </c>
       <c r="I8" s="10">
         <f>J9</f>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J8" s="10">
         <f t="shared" si="3"/>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="K8" s="10">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L8" s="10" t="str">
         <f t="shared" si="5"/>
@@ -1306,15 +1296,15 @@
       </c>
       <c r="I9" s="10">
         <f>J11</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J9" s="10">
         <f t="shared" si="3"/>
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="K9" s="10">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L9" s="10" t="str">
         <f t="shared" si="5"/>
@@ -1357,7 +1347,7 @@
         <v>27</v>
       </c>
       <c r="C10" s="14">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>20</v>
@@ -1368,7 +1358,7 @@
       </c>
       <c r="F10" s="10">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="G10" s="9">
         <f t="shared" si="1"/>
@@ -1376,11 +1366,11 @@
       </c>
       <c r="H10" s="9">
         <f t="shared" si="2"/>
-        <v>46353</v>
+        <v>46351</v>
       </c>
       <c r="I10" s="10">
         <f>J11</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J10" s="10">
         <f t="shared" si="3"/>
@@ -1438,27 +1428,27 @@
       </c>
       <c r="E11" s="10">
         <f>MAX(F9,F10)</f>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="F11" s="10">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G11" s="9">
         <f t="shared" si="1"/>
-        <v>46356</v>
+        <v>46352</v>
       </c>
       <c r="H11" s="9">
         <f t="shared" si="2"/>
-        <v>46358</v>
+        <v>46356</v>
       </c>
       <c r="I11" s="10">
         <f>MIN(J12,J13)</f>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="J11" s="10">
         <f t="shared" si="3"/>
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="K11" s="10">
         <f t="shared" si="4"/>
@@ -1512,27 +1502,27 @@
       </c>
       <c r="E12" s="10">
         <f>F11</f>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F12" s="10">
         <f t="shared" si="0"/>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G12" s="9">
         <f t="shared" si="1"/>
-        <v>46359</v>
+        <v>46357</v>
       </c>
       <c r="H12" s="9">
         <f t="shared" si="2"/>
-        <v>46364</v>
+        <v>46360</v>
       </c>
       <c r="I12" s="10">
         <f>J14</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J12" s="10">
         <f t="shared" si="3"/>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="K12" s="10">
         <f t="shared" si="4"/>
@@ -1586,27 +1576,27 @@
       </c>
       <c r="E13" s="10">
         <f>F11</f>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="F13" s="10">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G13" s="9">
         <f t="shared" si="1"/>
-        <v>46359</v>
+        <v>46357</v>
       </c>
       <c r="H13" s="9">
         <f t="shared" si="2"/>
-        <v>46363</v>
+        <v>46359</v>
       </c>
       <c r="I13" s="10">
         <f>J14</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J13" s="10">
         <f t="shared" si="3"/>
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="K13" s="10">
         <f t="shared" si="4"/>
@@ -1660,27 +1650,27 @@
       </c>
       <c r="E14" s="10">
         <f>MAX(F12,F13)</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F14" s="10">
         <f t="shared" si="0"/>
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="G14" s="9">
         <f t="shared" si="1"/>
-        <v>46365</v>
+        <v>46363</v>
       </c>
       <c r="H14" s="9">
         <f t="shared" si="2"/>
-        <v>46366</v>
+        <v>46364</v>
       </c>
       <c r="I14" s="10">
         <f>J15</f>
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="J14" s="10">
         <f t="shared" si="3"/>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="K14" s="10">
         <f t="shared" si="4"/>
@@ -1734,27 +1724,27 @@
       </c>
       <c r="E15" s="10">
         <f>F14</f>
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="F15" s="10">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="G15" s="9">
         <f t="shared" si="1"/>
-        <v>46367</v>
+        <v>46365</v>
       </c>
       <c r="H15" s="9">
         <f t="shared" si="2"/>
-        <v>46367</v>
+        <v>46365</v>
       </c>
       <c r="I15" s="10">
         <f>F15</f>
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J15" s="10">
         <f t="shared" si="3"/>
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="K15" s="10">
         <f t="shared" si="4"/>
@@ -1801,7 +1791,7 @@
       <c r="C17" s="6"/>
       <c r="D17" s="11">
         <f>MAX(F5:F15)</f>
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
@@ -1812,7 +1802,7 @@
       <c r="C18" s="6"/>
       <c r="D18" s="12">
         <f>MAX(H5:H15)</f>
-        <v>46367</v>
+        <v>46365</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
@@ -1832,9 +1822,7 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="15" t="s">
-        <v>44</v>
-      </c>
+      <c r="A23" s="15"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="L5:L15">

</xml_diff>